<commit_message>
Add Nikolas Moore credit watermark to web app and Excel template
</commit_message>
<xml_diff>
--- a/Goal Tracker Template.xlsx
+++ b/Goal Tracker Template.xlsx
@@ -708,10 +708,10 @@
     <from>
       <col>33</col>
       <colOff>0</colOff>
-      <row>0</row>
+      <row>3</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="2520000" cy="2160000"/>
+    <ext cx="2160000" cy="1800000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="3" name="Chart 3"/>
@@ -2265,7 +2265,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AP46"/>
+  <dimension ref="A1:AP47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -4815,6 +4815,13 @@
       <c r="AN46" s="4" t="n"/>
       <c r="AO46" s="4" t="n"/>
       <c r="AP46" s="4" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="1" t="inlineStr">
+        <is>
+          <t>© Nikolas Moore — Discipline Goal Tracker</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="16">

</xml_diff>